<commit_message>
Add Phase I appendix auto-generation (A/D/G) and best-practices rollout.
Auto-render appendices from Excel and sidebar meta into deliverable zips, with preflight predictions, batch per-site packages, CI package smoke, and Windows streamlit launcher.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/samples/phase1_devon_data.xlsx
+++ b/samples/phase1_devon_data.xlsx
@@ -699,7 +699,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Oil well site — drilled and abandoned / suspended</t>
+          <t>Oil well site — Devon 2017 reference</t>
         </is>
       </c>
       <c r="K2" t="inlineStr"/>
@@ -711,7 +711,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Informational interview with former site operator regarding waste disposal and infrastructure.</t>
+          <t>Informational interview with former operator regarding waste disposal and infrastructure.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -746,8 +746,10 @@
           <t>19-Jun-2004</t>
         </is>
       </c>
-      <c r="W2" t="n">
-        <v>710</v>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>710</t>
+        </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>

</xml_diff>